<commit_message>
EPBDS-9967 Remove $, thousands separators and K, M, B from numbers, which are not international and clash with $ step references
The workbooks keep their tables and write the same numbers in digits: the Bank Rating, Corporate Rating and
Tutorial 8 demo projects, every test copy of Bank Rating (also inside the ITEST zips), the Range-*,
CustomSpreadsheetInSpreadsheet and SimpleDTRangeAndArray workbooks, and EPBDS-7063, whose Date(2021,04,08)
is now Date(2021,4,8) because 08 is no longer read as decimal. In EPBDS-8323, SmartRules_IntRanges_Range now
checks that 77,99 matches 99, since a comma between digits always separates array elements.
</commit_message>
<xml_diff>
--- a/DEV/org.openl.rules.test/test-resources/functionality/CustomSpreadsheetInSpreadsheet.xlsx
+++ b/DEV/org.openl.rules.test/test-resources/functionality/CustomSpreadsheetInSpreadsheet.xlsx
@@ -2484,25 +2484,25 @@
          Components of the qualitative analysis are monitoring of bank-counterparty’s ratings assigned by international rating agencies, the existence and nature of the bank's credit history, current level of relationships with the bank, its shareholders and management, the business reputational analysis of the bank, monitoring of relations with a financial supervisory authority.</t>
   </si>
   <si>
-    <t>&lt; 8K</t>
-  </si>
-  <si>
-    <t>[8K .. 100K)</t>
-  </si>
-  <si>
-    <t>&gt;= 100K</t>
-  </si>
-  <si>
-    <t>&lt; 1K</t>
-  </si>
-  <si>
-    <t>[1K .. 10K)</t>
-  </si>
-  <si>
-    <t>&gt;= 10K</t>
-  </si>
-  <si>
-    <t>&lt; 2K</t>
+    <t>&lt; 8000</t>
+  </si>
+  <si>
+    <t>[8000 .. 100000)</t>
+  </si>
+  <si>
+    <t>&gt;= 100000</t>
+  </si>
+  <si>
+    <t>&lt; 1000</t>
+  </si>
+  <si>
+    <t>[1000 .. 10000)</t>
+  </si>
+  <si>
+    <t>&gt;= 10000</t>
+  </si>
+  <si>
+    <t>&lt; 2000</t>
   </si>
   <si>
     <t>&gt;= 600</t>
@@ -2514,19 +2514,19 @@
     <t>&lt; 200</t>
   </si>
   <si>
-    <t>&gt; 1K</t>
-  </si>
-  <si>
-    <t>[200 .. 1K]</t>
+    <t>&gt; 1000</t>
+  </si>
+  <si>
+    <t>[200 .. 1000]</t>
   </si>
   <si>
     <t>DE</t>
   </si>
   <si>
-    <t>[2K .. 30K)</t>
-  </si>
-  <si>
-    <t>&gt;= 30K</t>
+    <t>[2000 .. 30000)</t>
+  </si>
+  <si>
+    <t>&gt;= 30000</t>
   </si>
   <si>
     <t>BE</t>

</xml_diff>